<commit_message>
Remove customer branding from public demo
Rebrand the app as Meihao Airlines, replace carrier-specific mock data with generic synthetic markers, refresh knowledge snapshots, documentation and workbook assets.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/templates/city-airport-mapping.xlsx
+++ b/data/templates/city-airport-mapping.xlsx
@@ -6347,7 +6347,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>城市／機場地理對照範本；不是已核驗的 DEMO 營運航網。</t>
+          <t>城市／機場地理對照範本；不代表任何航空公司的實際營運航網。</t>
         </is>
       </c>
     </row>
@@ -6403,14 +6403,14 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>RouteReferences 可空白；即使填入也只是獨立參考，不建立 DEMO 自營／可售資格，不更動合成 flight generator。</t>
+          <t>RouteReferences 可空白；填入的資料僅供獨立參考，不建立可售資格或更動合成航班生成器。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>RouteReferences 行銷與實際營運皆必須 DEMO；不接受 AE、夥伴航空或共掛替代。</t>
+          <t>路線參考不驗證航空公司的實際營運資格。</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>範本不含公式、巨集、樣本 DEMO 航線或個人資料；整份 Excel 不送往 LLM／向量庫。</t>
+          <t>範本不含公式、巨集、樣本航空公司航線或個人資料；整份 Excel 不送往 LLM／向量庫。</t>
         </is>
       </c>
     </row>

</xml_diff>